<commit_message>
Renombra salario a 'Ricardo' y registra pago del 01/10/2026 (comprobante 20614541, ELI)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KbxaieUYjEnXLJEuZbCTyf
</commit_message>
<xml_diff>
--- a/Registro_Pagos_Fijos_Octubre_2026_OliEli.xlsx
+++ b/Registro_Pagos_Fijos_Octubre_2026_OliEli.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Salario Ricardo José (Edición y Creador de Contenido)</t>
+          <t>Salario Ricardo (Edición y Creador de Contenido)</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
@@ -931,14 +931,26 @@
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H12" s="9" t="n"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>20614541</t>
+        </is>
+      </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>ELI</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1340,7 +1352,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Salario Ricardo José (Edición y Creador de Contenido)</t>
+          <t>Salario Ricardo (Edición y Creador de Contenido)</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">

</xml_diff>

<commit_message>
Mueve pago de Ricardo (comprobante 20614541) a la fila del 15 de septiembre
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KbxaieUYjEnXLJEuZbCTyf
</commit_message>
<xml_diff>
--- a/Registro_Pagos_Fijos_Octubre_2026_OliEli.xlsx
+++ b/Registro_Pagos_Fijos_Octubre_2026_OliEli.xlsx
@@ -931,26 +931,14 @@
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>20614541</t>
-        </is>
-      </c>
+      <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J12" s="9" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="K12" s="9" t="inlineStr">
-        <is>
-          <t>ELI</t>
-        </is>
-      </c>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Agrega Excel de septiembre 2026 y actualiza Excel de octubre (sin logo, con cierre de mes)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KbxaieUYjEnXLJEuZbCTyf
</commit_message>
<xml_diff>
--- a/Registro_Pagos_Fijos_Octubre_2026_OliEli.xlsx
+++ b/Registro_Pagos_Fijos_Octubre_2026_OliEli.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,12 +30,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
@@ -52,6 +47,14 @@
     <font>
       <i val="1"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008B0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -82,7 +85,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -104,11 +107,16 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -116,40 +124,48 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -516,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -535,1048 +551,1089 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OLI &amp; ELI · TU BARBERÍA</t>
+          <t>REGISTRO DE PAGOS FIJOS - OCTUBRE 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>REGISTRO DE PAGOS FIJOS - OCTUBRE 2026</t>
+          <t>Pagos fijos mensuales recurrentes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Pagos fijos mensuales recurrentes — Encargada Área Contable: OLIVA RUIZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Fecha Máxima de Pago</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Detalle de Pago</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Monto ($)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Comisión ($)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Valor Total ($)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Destinatario</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Banco / Entidad</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>N° de Comprobante</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Forma de Pago</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Fecha de Pago / Cancelación</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Fecha Máxima de Pago</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Detalle de Pago</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Monto ($)</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Comisión ($)</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Valor Total ($)</t>
-        </is>
+          <t>30 de cada mes</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Internet Local Xtrim</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E4" s="7">
+        <f>C4+D4</f>
+        <v/>
       </c>
       <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Destinatario</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Banco / Entidad</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>N° de Comprobante</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Forma de Pago</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Fecha de Pago / Cancelación</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Responsable</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>30 de cada mes</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Internet Local Xtrim</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="E5" s="8">
-        <f>C5+D5</f>
-        <v/>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Oliva Ruiz (CI: 1722594346)
 Cta: Débito directo</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>01 de cada mes</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Arriendo local</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C5" s="10" t="n">
         <v>700</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="12">
-        <f>C6+D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="E5" s="11">
+        <f>C5+D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Laura Narváez (CI: 1705406013)
 Cta: 3249401800</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>01 de cada mes</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Limpieza local</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="8">
-        <f>C7+D7</f>
-        <v/>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="E6" s="7">
+        <f>C6+D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Esperanza Lastra (CI: 10018739246)
 Cta: 2204907756</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>01 de cada mes</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Aplicación Fresha</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C7" s="10" t="n">
         <v>3.95</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D7" s="10" t="n">
         <v>0.41</v>
       </c>
-      <c r="E8" s="12">
-        <f>C8+D8</f>
-        <v/>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="E7" s="11">
+        <f>C7+D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Rocío Elizabeth Ruiz (CI: 1719052431)
 Cta: 4120101340 76</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Coop. Alianza del
 Valle</t>
         </is>
       </c>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>01 de cada mes</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Salario Elizabeth (Eli)</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="8">
-        <f>C9+D9</f>
-        <v/>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="E8" s="7">
+        <f>C8+D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Rocío Elizabeth Ruiz (CI: 1719052431)
 Cta: 4775767300</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>01 de cada mes</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Salario Oliva (Oli)</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C9" s="10" t="n">
         <v>300</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="12">
-        <f>C10+D10</f>
-        <v/>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E9" s="11">
+        <f>C9+D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Oliva Esperanza Ruiz (CI: 1722594346)
 Cta: 7700305630</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="inlineStr">
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>01 de cada mes</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Recepcionista/Cajera
 (Mayerly)</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="8">
-        <f>C11+D11</f>
-        <v/>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="E10" s="7">
+        <f>C10+D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Mayerly Santistevan (CI: 2350981672)
 Cta: 2207337955</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>01 de cada mes</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Salario Ricardo (Edición y Creador de Contenido)</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C11" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="12">
-        <f>C12+D12</f>
-        <v/>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="E11" s="11">
+        <f>C11+D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Ricardo Alquinga (CI: 1727069534)
 Cta: 2209846247</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="inlineStr">
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="J11" s="8" t="n"/>
+      <c r="K11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>04 de cada mes</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Pago de luz</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Empresa Eléctrica (CI: —)
 Cta: —</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Empresa Eléctrica</t>
         </is>
       </c>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>05 de cada mes</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Productos Level3</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Jaqueline Pinto (CI: 1707128136)
 Cta: 2205468517</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="J13" s="8" t="n"/>
+      <c r="K13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>08 de cada mes</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Pago de agua</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>EPMAPS (Agua de Quito) (CI: —)
 Cta: —</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>EPMAPS</t>
         </is>
       </c>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>10 de cada mes</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>ChatGPT</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C15" s="10" t="n">
         <v>19.99</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D15" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E16" s="12">
-        <f>C16+D16</f>
-        <v/>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="E15" s="11">
+        <f>C15+D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Oliva Ruiz (CI: 1722594346)
 Cta: Débito directo</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Banca Móvil (local)</t>
         </is>
       </c>
-      <c r="H16" s="9" t="n"/>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Débito</t>
         </is>
       </c>
-      <c r="J16" s="9" t="n"/>
-      <c r="K16" s="9" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="J15" s="8" t="n"/>
+      <c r="K15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>10 de cada mes</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Préstamo Escuela Alianza</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>898.39</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D16" s="6" t="n">
         <v>0.41</v>
       </c>
-      <c r="E17" s="8">
-        <f>C17+D17</f>
-        <v/>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="E16" s="7">
+        <f>C16+D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Rocío Elizabeth Ruiz Lastra (CI:
 1706663364)
 Cta: 4120101340 76</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Coop. Alianza del
 Valle</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>11 de cada mes</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Amazon - Alexa</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C17" s="10" t="n">
         <v>3.99</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D17" s="10" t="n">
         <v>0.8</v>
       </c>
-      <c r="E18" s="12">
-        <f>C18+D18</f>
-        <v/>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="E17" s="11">
+        <f>C17+D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Amazon (por confirmar) (CI: —)
 Cta: —</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Por confirmar</t>
         </is>
       </c>
-      <c r="H18" s="9" t="n"/>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Débito</t>
         </is>
       </c>
-      <c r="J18" s="9" t="n"/>
-      <c r="K18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="J17" s="8" t="n"/>
+      <c r="K17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>15 de cada mes</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Limpieza local</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C18" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="8">
-        <f>C19+D19</f>
-        <v/>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="E18" s="7">
+        <f>C18+D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Esperanza Lastra (CI: 10018739246)
 Cta: 2204907756</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>15 de cada mes</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Salario Elizabeth (Eli)</t>
         </is>
       </c>
-      <c r="C20" s="11" t="n">
+      <c r="C19" s="10" t="n">
         <v>300</v>
       </c>
-      <c r="D20" s="11" t="n">
+      <c r="D19" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="12">
-        <f>C20+D20</f>
-        <v/>
-      </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="E19" s="11">
+        <f>C19+D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Rocío Elizabeth Ruiz (CI: 1719052431)
 Cta: 4775767300</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H20" s="9" t="n"/>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="H19" s="8" t="n"/>
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J20" s="9" t="n"/>
-      <c r="K20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="J19" s="8" t="n"/>
+      <c r="K19" s="8" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>15 de cada mes</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Salario Oliva (Oli)</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C20" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="8">
-        <f>C21+D21</f>
-        <v/>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="E20" s="7">
+        <f>C20+D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Oliva Esperanza Ruiz (CI: 1722594346)
 Cta: 7700305630</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>15 de cada mes</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Recepcionista/Cajera
 (Mayerly)</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
+      <c r="C21" s="10" t="n">
         <v>300</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D21" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="12">
-        <f>C22+D22</f>
-        <v/>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E21" s="11">
+        <f>C21+D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Mayerly Santistevan (CI: 2350981672)
 Cta: 2207337955</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="9" t="inlineStr">
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J22" s="9" t="n"/>
-      <c r="K22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="J21" s="8" t="n"/>
+      <c r="K21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>15 de cada mes</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Salario Ricardo (Edición y Creador de Contenido)</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C22" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D22" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="8">
-        <f>C23+D23</f>
-        <v/>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="E22" s="7">
+        <f>C22+D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Ricardo Alquinga (CI: 1727069534)
 Cta: 2209846247</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>15 de cada mes</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Arriendo Escuela</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
+      <c r="C23" s="10" t="n">
         <v>500</v>
       </c>
-      <c r="D24" s="11" t="n">
+      <c r="D23" s="10" t="n">
         <v>0.41</v>
       </c>
-      <c r="E24" s="12">
-        <f>C24+D24</f>
-        <v/>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E23" s="11">
+        <f>C23+D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Rodrigo Mora (CI: 1706663364)
 Cta: 12004033537 (Produbanco)</t>
         </is>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>Produbanco</t>
         </is>
       </c>
-      <c r="H24" s="9" t="n"/>
-      <c r="I24" s="9" t="inlineStr">
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J24" s="9" t="n"/>
-      <c r="K24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="J23" s="8" t="n"/>
+      <c r="K23" s="8" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>18 de cada mes</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Préstamo Alianza del Valle</t>
         </is>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C24" s="6" t="n">
         <v>601.65</v>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D24" s="6" t="n">
         <v>0.41</v>
       </c>
-      <c r="E25" s="8">
-        <f>C25+D25</f>
-        <v/>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="E24" s="7">
+        <f>C24+D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Oliva Ruiz (CI: 1722594346)
 Cta: 4120100934 18</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Coop. Alianza del
 Valle</t>
         </is>
       </c>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Transferencia</t>
         </is>
       </c>
-      <c r="J25" s="5" t="n"/>
-      <c r="K25" s="5" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>19 de cada mes</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Préstamo Banco Pichincha</t>
         </is>
       </c>
-      <c r="C26" s="11" t="n">
+      <c r="C25" s="10" t="n">
         <v>657.08</v>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D25" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="12">
-        <f>C26+D26</f>
-        <v/>
-      </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="E25" s="11">
+        <f>C25+D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Oliva Ruiz (CI: 1722594346)
 Cta: Débito directo</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H26" s="9" t="n"/>
-      <c r="I26" s="9" t="inlineStr">
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>Débito</t>
         </is>
       </c>
-      <c r="J26" s="9" t="n"/>
-      <c r="K26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="J25" s="8" t="n"/>
+      <c r="K25" s="8" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>21 de cada mes</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Aplicación CapCut</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n">
+      <c r="C26" s="6" t="n">
         <v>6.99</v>
       </c>
-      <c r="D27" s="7" t="n">
+      <c r="D26" s="6" t="n">
         <v>1.4</v>
       </c>
-      <c r="E27" s="8">
-        <f>C27+D27</f>
-        <v/>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="E26" s="7">
+        <f>C26+D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Oliva Ruiz (CI: 1722594346)
 Cta: Débito directo</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>Banco Pichincha</t>
         </is>
       </c>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Débito</t>
         </is>
       </c>
-      <c r="J27" s="5" t="n"/>
-      <c r="K27" s="5" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="13" t="n"/>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>TOTAL GASTOS FIJOS MENSUALES</t>
         </is>
       </c>
-      <c r="C28" s="14">
-        <f>SUM(C5:C27)</f>
-        <v/>
-      </c>
-      <c r="D28" s="14">
-        <f>SUM(D5:D27)</f>
-        <v/>
-      </c>
-      <c r="E28" s="14">
-        <f>SUM(E5:E27)</f>
-        <v/>
-      </c>
-      <c r="F28" s="13" t="n"/>
-      <c r="G28" s="13" t="n"/>
-      <c r="H28" s="13" t="n"/>
-      <c r="I28" s="13" t="n"/>
-      <c r="J28" s="13" t="n"/>
-      <c r="K28" s="13" t="n"/>
-    </row>
-    <row r="29" ht="35" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="C27" s="13">
+        <f>SUM(C4:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="13">
+        <f>SUM(D4:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="13">
+        <f>SUM(E4:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>OBSERVACIÓN: existen pagos que se debitan mes a mes de la Cooperativa Cooprogreso. Hay que estar pendientes de ese estado de cuenta en el mes de diciembre, para incluirlo en el cierre del año y saber cuánto queda pendiente de pagar y cuánto queda existente para su respectivo cobro hasta el mes de marzo.</t>
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>CIERRE DE MES — OCTUBRE 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Certificamos que los pagos fijos del mes detallados en este registro han sido revisados y conciliados con sus respectivos comprobantes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="17" t="n"/>
+      <c r="F35" s="17" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>MAYERLY SANTISTEVAN</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="inlineStr">
+        <is>
+          <t>ELIZABETH RUIZ</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Fecha de cierre: ____ / ____ / ________</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>Asistente</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>Administradora</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A30:K30"/>
     <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A28:K28"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A29:K29"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A31:K31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>

</xml_diff>